<commit_message>
Align the reproduction package with the submitted figures and Supporting Information.
Figure 1 uses the current assignment layout, Figure 2 uses the submitted reference numbers, and the package now regenerates S4 Fig and SI_5 table and includes S1 Figure 1 and the current SI_3 workbook.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/supporting_information/SI_2_MethodsTable.xlsx
+++ b/supporting_information/SI_2_MethodsTable.xlsx
@@ -6,7 +6,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="44800" windowHeight="22800" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1 Table" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SI_2 table" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -305,7 +305,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -445,6 +445,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -834,21 +843,21 @@
     <row r="1">
       <c r="A1" s="50" t="inlineStr">
         <is>
-          <t>S2 Table. Comprehensive survey of 60 computational methods for cell reprogramming (2013 to 2026), with explicitness class and V/U descriptor columns</t>
+          <t>SI_2 table. Comprehensive survey of 60 computational methods for cell reprogramming (2013 to 2026), with explicitness class, validation code, and uncertainty code</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="51" t="inlineStr">
         <is>
-          <t>Columns are organized into seven thematic blocks described below. Block 3 includes explicitness class assignments following Section 3 and Table 1; full class definitions and V0, V4 / U0, U4 codes are in Supporting Information S1 (SI_1_FourClassTaxonomy.pdf).</t>
+          <t>Columns are organized into seven thematic blocks described below. Block 3 includes explicitness class assignments following Section 3; full class definitions and V0 to V4 and U0 to U4 codes are in Supporting Information S1 (SI_1_FourClassTaxonomy.pdf).</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="48" customHeight="1" s="18">
       <c r="A3" s="52" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-28 (v2). Extends the original 51-method audit with 5 peer-reviewed 2025 to 2026 methods: REVIVE, CANDiT, SwitchTFI, Atlas-guided T-cell programming, REPROcode. Reprogram-Seq (PMID 31216470) inserted among 2019 methods (18 Sep 2026). Iterative TF screening (PMID 40494892) inserted among 2025 methods (18 Sep 2026). TF Atlas (PMID 36608654) inserted among 2023 methods (18 Sep 2026). Briggs combinatorial TF landscape (PMID 42314680) inserted among 2026 methods (18 Sep 2026). TRAPT dropped 18 Sep 2026 (M2 fail; retained on the eligibility log). Explicitness classes are taken from reprogramming_methods_4_level_classification.xlsx.</t>
+          <t>Catalogue passes. The first audit (10 December 2025) covered 51 methods published from 2013 to 2025; published web-tool addresses were opened on 10 to 11 December 2025. On 4 May 2026, five methods were added: CANDiT (2025), REVIVE (2025), SwitchTFI (2025), Atlas-guided T-cell programming (2026), and REPROcode (2026). On 18 September 2026, four methods were added: Reprogram-Seq (2019), TF Atlas (2023), Iterative TF screening (2025), and Briggs combinatorial TF landscape (2026).</t>
         </is>
       </c>
     </row>
@@ -862,21 +871,21 @@
     <row r="5" ht="23" customHeight="1" s="18">
       <c r="A5" s="51" t="inlineStr">
         <is>
-          <t>Block 2 : Biological Scope. Data Scale: input data granularity can be Bulk, Single-cell, Both, or Model-based (operates on a curated network model without omics input). Reprogramming Modality: one or more of four canonical types, semicolon-separated types Indirect reprogramming (to pluripotency), Directed differentiation, Transdifferentiation, Phenotype reprogramming. Intervention Type: TF, transcription factors only; TF+, transcription factors together with other molecular targets (signaling proteins, kinases, miRNAs, epigenetic modifiers); SM, small molecules or chemical compounds.</t>
+          <t>Block 2 : Biological Scope. Data Scale: input data granularity can be Bulk, Single-cell, Both, or Model-based (operates on a curated network model without omics input). Reprogramming Setting: one or more of four canonical types, semicolon-separated types Indirect reprogramming (to pluripotency), Directed differentiation, Transdifferentiation, Phenotype reprogramming. Intervention Type: TF, transcription factors only; TF+, transcription factors together with other molecular targets (signaling proteins, kinases, miRNAs, epigenetic modifiers); SM, small molecules or chemical compounds.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="49" customHeight="1" s="18">
+    <row r="6" ht="68" customHeight="1" s="18">
       <c r="A6" s="51" t="inlineStr">
         <is>
-          <t>Block 3: Methodological Taxonomy. Input Data: semicolon-separated data-type tags include GRN (gene regulatory network topology), BN (Boolean network model), Bulk RNA-seq data, scRNA-seq data, ATAC-seq data, ChIP-seq data, Hi-C data, TF motifs, PPI (protein, protein interaction network), ODE (ordinary differential equation model), Perturbation signatures (subtyped as LINCS, PLATE-seq, ChemPert, NCPC, or sciPlex), Proteomics (subtyped as RPPA, phosphoproteomics, or CyTOF). Inverse Design Level: compact code for the four-level taxonomy (C0 = target-feature discovery; C1 = network-informed inverse-design heuristic; C2 (signature) = proxy inverse design via signature/state matching; C2 (network) = proxy inverse design via network propagation; C3 = explicit model-based inverse intervention). Level detail: for C3 methods, operator sub-family (3A, 3F) and model provenance; for borderline placements, a brief note; otherwise em dash. Mathematical Framework: general tag optionally followed by a colon and specific subtype. General tags include Boolean network (subtypes: Probabilistic BN), ODE, Static network (subtypes: GRN influence, PageRank, Multi-omics integration), Information theory (subtypes: JSD, MMI), Machine learning (subtypes: Random forest, KNN, SVM, Linear regression, Logistic regression), Deep learning (subtypes: GNN, GAT, MLP, Deep RL), Signature matching (subtypes: GSEA, C1 distance, correlation), Control theory (subtypes: FVS, MDP, Optimal control, Feedback design), Computational algebra, Energy landscape, Signal propagation. Target Prioritization: formatted as Output type; scoring metric. Output types include Ranked list, Minimal control sets, Control policy, Filtered sets, None. Approach: Dynamic (explicit temporal simulation of network state transitions) or Static (no dynamical simulation). Validation code (V0, V4): compact validation-evidence tier (V0 conceptual; V1 retrospective recovery; V2 held-out perturbation prediction; V3 prospective in vitro, including functional endpoints recorded in the Validation column; V4 in vivo or cross-lab). Uncertainty (U0, U4): uncertainty and calibration reporting tier (U0 none reported; U1 ranking only; U2 local stability; U3 documented sensitivity; U4 calibrated/OOD checks). Validation code (V0, V4): compact validation-evidence tier (V0 conceptual; V1 retrospective recovery; V2 held-out perturbation prediction; V3 prospective in vitro, including functional endpoints recorded in the Validation column; V4 in vivo or cross-lab). Uncertainty (U0, U4): uncertainty and calibration reporting tier (U0 none reported; U1 ranking only; U2 local stability; U3 documented sensitivity; U4 calibrated/OOD checks). Validation code (V0, V4): compact validation-evidence tier (V0 conceptual; V1 retrospective recovery; V2 held-out perturbation prediction; V3 prospective in vitro, including functional endpoints recorded in the Validation column; V4 in vivo or cross-lab). Uncertainty (U0, U4): uncertainty and calibration reporting tier (U0 none reported; U1 ranking only; U2 local stability; U3 documented sensitivity; U4 calibrated/OOD checks).</t>
+          <t>Block 3: Methodological Taxonomy. Input Data: semicolon-separated data-type tags include GRN (gene regulatory network topology), BN (Boolean network model), Bulk RNA-seq data, scRNA-seq data, ATAC-seq data, ChIP-seq data, Hi-C data, TF motifs, PPI (protein-protein interaction network), ODE (ordinary differential equation model), Perturbation signatures (subtyped as LINCS, PLATE-seq, ChemPert, NCPC, or sciPlex), Proteomics (subtyped as RPPA, phosphoproteomics, or CyTOF). Explicitness class: compact code for the four-class taxonomy (C0 = target-feature discovery; C1 = network-informed inverse-design heuristic; C2 (signature) = proxy inverse design via signature/state matching; C2 (network) = proxy inverse design via network propagation; C3 = explicit model-based inverse intervention). Class detail: for C3 methods, operator sub-family (3A to 3F) and model provenance; for borderline placements, a brief note; otherwise a hyphen (-). Mathematical Framework: general tag optionally followed by a colon and specific subtype. General tags include Boolean network (subtypes: Probabilistic BN), ODE, Static network (subtypes: GRN influence, PageRank, Multi-omics integration), Information theory (subtypes: JSD, MMI), Machine learning (subtypes: Random forest, KNN, SVM, Linear regression, Logistic regression), Deep learning (subtypes: GNN, GAT, MLP, Deep RL), Signature matching (subtypes: GSEA, L1 distance, correlation), Control theory (subtypes: FVS, MDP, Optimal control, Feedback design), Computational algebra, Energy landscape, Signal propagation. Target Prioritization: formatted as Output type; scoring metric. Output types include Ranked list, Minimal control sets, Control policy, Filtered sets, None. Approach: Dynamic (explicit temporal simulation of network state transitions) or Static (no dynamical simulation).</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1" s="18">
+    <row r="7" ht="90" customHeight="1" s="18">
       <c r="A7" s="51" t="inlineStr">
         <is>
-          <t>Block 4 : Validation &amp; Benchmarking. Validation: Biological problem(s) used to validate method. Types can be In silico, In vitro, In vivo, or combinations thereof. Qualifiers used are "reproduced" (recovery of previously known reprogramming targets), "novel" (new experimental validation), or reproduced + novel. The suffix "BN" after a system name indicates that validation was performed on a Boolean network model. Benchmarked Against: "None" or a semicolon-separated list of other computational cell reprogramming / cell-fate design methods in this survey (PubMed identifiers when available). Include only head-to-head comparisons to methods whose primary output is a reprogramming intervention proposal (ranked TFs, cocktails, perturbagens, or control policies toward a target state). Do not list trajectory-driver tools (e.g. CellRank, spliceJAC, DrivAER), TR-recovery or motif-enrichment tools (e.g. Lisa, ChEA3), perturbation-response predictors (e.g. GEARS, scGen), aging databases or clocks (e.g. DrugAge), or experimental/screening baselines, even when the original paper reports such benchmarks; note those under Validation instead. Example: SwitchTFI is benchmarked against CellRank in its publication, but CellRank is not a cell reprogramming method in this column's sense, so the entry is "None".</t>
+          <t>Block 4 : Validation &amp; Benchmarking. Validation: Biological problem(s) used to validate method. Types can be In silico, In vitro, In vivo, or combinations thereof. Qualifiers used are "reproduced" (recovery of previously known reprogramming targets), "novel" (new experimental validation), or reproduced + novel. The suffix "BN" after a system name indicates that validation was performed on a Boolean network model. Validation code (V0 to V4): compact validation-evidence tier (V0 conceptual; V1 retrospective recovery; V2 held-out perturbation prediction; V3 prospective in vitro, including functional endpoints recorded in the Validation column; V4 in vivo or cross-lab). Uncertainty (U0 to U4): uncertainty and calibration reporting tier (U0 none reported; U1 ranking only; U2 local stability; U3 documented sensitivity; U4 calibrated/OOD checks). Benchmarked Against: "None" or a semicolon-separated list of other computational cell reprogramming / cell-fate design methods in this survey (PubMed identifiers when available). Include only head-to-head comparisons to methods whose primary output is a reprogramming intervention proposal (ranked TFs, cocktails, perturbagens, or control policies toward a target state). Do not list trajectory-driver tools (e.g. CellRank, spliceJAC, DrivAER), TR-recovery or motif-enrichment tools (e.g. Lisa, ChEA3), perturbation-response predictors (e.g. GEARS, scGen), aging databases or clocks (e.g. DrugAge), or experimental/screening baselines, even when the original paper reports such benchmarks; note those under Validation instead. Example: SwitchTFI is benchmarked against CellRank in its publication, but CellRank is not a cell reprogramming method in this column's sense, so the entry is "None".</t>
         </is>
       </c>
     </row>
@@ -901,6 +910,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="22" customHeight="1" s="18">
       <c r="A12" s="31" t="inlineStr">
         <is>
@@ -932,16 +942,20 @@
           <t>Block 4 : Validation &amp; Benchmarking</t>
         </is>
       </c>
-      <c r="O12" s="48" t="n"/>
-      <c r="P12" s="32" t="n"/>
-      <c r="Q12" s="33" t="n"/>
-      <c r="R12" s="49" t="n"/>
+      <c r="O12" s="47" t="n"/>
+      <c r="P12" s="47" t="n"/>
+      <c r="Q12" s="48" t="n"/>
+      <c r="R12" s="34" t="inlineStr">
+        <is>
+          <t>Block 5 : Availability</t>
+        </is>
+      </c>
       <c r="S12" s="31" t="inlineStr">
         <is>
           <t>Block 6 : Resources</t>
         </is>
       </c>
-      <c r="T12" s="33" t="n"/>
+      <c r="T12" s="48" t="n"/>
       <c r="U12" s="34" t="inlineStr">
         <is>
           <t>Block 7 : Reference</t>
@@ -976,7 +990,7 @@
       </c>
       <c r="F13" s="36" t="inlineStr">
         <is>
-          <t>Reprogramming Modality</t>
+          <t>Reprogramming Setting</t>
         </is>
       </c>
       <c r="G13" s="37" t="inlineStr">
@@ -1157,7 +1171,7 @@
         </is>
       </c>
       <c r="U14" s="42" t="n">
-        <v>71</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" ht="45" customHeight="1" s="18">
@@ -1262,7 +1276,7 @@
         </is>
       </c>
       <c r="U15" s="46" t="n">
-        <v>70</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" ht="45" customHeight="1" s="18">
@@ -1367,7 +1381,7 @@
         </is>
       </c>
       <c r="U16" s="42" t="n">
-        <v>82</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" ht="45" customHeight="1" s="18">
@@ -1472,7 +1486,7 @@
         </is>
       </c>
       <c r="U17" s="46" t="n">
-        <v>62</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" ht="45" customHeight="1" s="18">
@@ -1578,7 +1592,7 @@
         </is>
       </c>
       <c r="U18" s="42" t="n">
-        <v>21</v>
+        <v>48</v>
       </c>
     </row>
     <row r="19" ht="45" customHeight="1" s="18">
@@ -1683,7 +1697,7 @@
         </is>
       </c>
       <c r="U19" s="46" t="n">
-        <v>81</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" ht="45" customHeight="1" s="18">
@@ -1788,7 +1802,7 @@
         </is>
       </c>
       <c r="U20" s="42" t="n">
-        <v>34</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" ht="45" customHeight="1" s="18">
@@ -1893,7 +1907,7 @@
         </is>
       </c>
       <c r="U21" s="46" t="n">
-        <v>55</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" ht="45" customHeight="1" s="18">
@@ -1998,7 +2012,7 @@
         </is>
       </c>
       <c r="U22" s="42" t="n">
-        <v>26</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1" s="18">
@@ -2105,7 +2119,7 @@
         </is>
       </c>
       <c r="U23" s="46" t="n">
-        <v>72</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" ht="45" customHeight="1" s="18">
@@ -2210,7 +2224,7 @@
         </is>
       </c>
       <c r="U24" s="42" t="n">
-        <v>73</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" ht="45" customHeight="1" s="18">
@@ -2315,7 +2329,7 @@
         </is>
       </c>
       <c r="U25" s="46" t="n">
-        <v>74</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1" s="18">
@@ -2420,7 +2434,7 @@
         </is>
       </c>
       <c r="U26" s="42" t="n">
-        <v>67</v>
+        <v>114</v>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1" s="18">
@@ -2525,7 +2539,7 @@
         </is>
       </c>
       <c r="U27" s="46" t="n">
-        <v>61</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" ht="45" customHeight="1" s="18">
@@ -2630,7 +2644,7 @@
         </is>
       </c>
       <c r="U28" s="42" t="n">
-        <v>63</v>
+        <v>108</v>
       </c>
     </row>
     <row r="29" ht="45" customHeight="1" s="18">
@@ -2735,7 +2749,7 @@
         </is>
       </c>
       <c r="U29" s="46" t="n">
-        <v>31</v>
+        <v>59</v>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1" s="18">
@@ -2840,7 +2854,7 @@
         </is>
       </c>
       <c r="U30" s="42" t="n">
-        <v>75</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31" ht="45" customHeight="1" s="18">
@@ -2945,7 +2959,7 @@
         </is>
       </c>
       <c r="U31" s="46" t="n">
-        <v>42</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32" ht="45" customHeight="1" s="18">
@@ -3050,7 +3064,7 @@
         </is>
       </c>
       <c r="U32" s="42" t="n">
-        <v>76</v>
+        <v>121</v>
       </c>
     </row>
     <row r="33" ht="45" customHeight="1" s="18">
@@ -3157,7 +3171,7 @@
         </is>
       </c>
       <c r="U33" s="46" t="n">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="34" ht="45" customHeight="1" s="18">
@@ -3259,7 +3273,9 @@
           <t>3/5</t>
         </is>
       </c>
-      <c r="U34" s="42" t="n"/>
+      <c r="U34" s="42" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="35" ht="45" customHeight="1" s="18">
       <c r="A35" s="43" t="inlineStr">
@@ -3274,7 +3290,7 @@
       </c>
       <c r="C35" s="44" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PMID: 34141873</t>
+          <t>PMID: 34141873</t>
         </is>
       </c>
       <c r="D35" s="45" t="inlineStr">
@@ -3363,7 +3379,7 @@
         </is>
       </c>
       <c r="U35" s="46" t="n">
-        <v>60</v>
+        <v>123</v>
       </c>
     </row>
     <row r="36" ht="45" customHeight="1" s="18">
@@ -3468,7 +3484,7 @@
         </is>
       </c>
       <c r="U36" s="42" t="n">
-        <v>77</v>
+        <v>122</v>
       </c>
     </row>
     <row r="37" ht="45" customHeight="1" s="18">
@@ -3573,7 +3589,7 @@
         </is>
       </c>
       <c r="U37" s="46" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38" ht="45" customHeight="1" s="18">
@@ -3678,7 +3694,7 @@
         </is>
       </c>
       <c r="U38" s="42" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
     </row>
     <row r="39" ht="45" customHeight="1" s="18">
@@ -3784,7 +3800,7 @@
         </is>
       </c>
       <c r="U39" s="46" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" ht="45" customHeight="1" s="18">
@@ -3800,7 +3816,7 @@
       </c>
       <c r="C40" s="40" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PMID: 34244796 </t>
+          <t>PMID: 34244796</t>
         </is>
       </c>
       <c r="D40" s="41" t="inlineStr">
@@ -3889,7 +3905,7 @@
         </is>
       </c>
       <c r="U40" s="42" t="n">
-        <v>25</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" ht="45" customHeight="1" s="18">
@@ -3994,7 +4010,7 @@
         </is>
       </c>
       <c r="U41" s="46" t="n">
-        <v>56</v>
+        <v>105</v>
       </c>
     </row>
     <row r="42" ht="45" customHeight="1" s="18">
@@ -4099,7 +4115,7 @@
         </is>
       </c>
       <c r="U42" s="42" t="n">
-        <v>48</v>
+        <v>63</v>
       </c>
     </row>
     <row r="43" ht="45" customHeight="1" s="18">
@@ -4205,7 +4221,7 @@
         </is>
       </c>
       <c r="U43" s="46" t="n">
-        <v>23</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" ht="45" customHeight="1" s="18">
@@ -4312,7 +4328,7 @@
         </is>
       </c>
       <c r="U44" s="42" t="n">
-        <v>41</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45" ht="45" customHeight="1" s="18">
@@ -4417,7 +4433,7 @@
         </is>
       </c>
       <c r="U45" s="46" t="n">
-        <v>65</v>
+        <v>115</v>
       </c>
     </row>
     <row r="46" ht="45" customHeight="1" s="18">
@@ -4522,7 +4538,7 @@
         </is>
       </c>
       <c r="U46" s="42" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
     </row>
     <row r="47" ht="45" customHeight="1" s="18">
@@ -4627,7 +4643,7 @@
         </is>
       </c>
       <c r="U47" s="46" t="n">
-        <v>68</v>
+        <v>106</v>
       </c>
     </row>
     <row r="48" ht="45" customHeight="1" s="18">
@@ -4732,7 +4748,7 @@
         </is>
       </c>
       <c r="U48" s="42" t="n">
-        <v>53</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49" ht="45" customHeight="1" s="18">
@@ -4837,7 +4853,7 @@
         </is>
       </c>
       <c r="U49" s="46" t="n">
-        <v>59</v>
+        <v>119</v>
       </c>
     </row>
     <row r="50" ht="45" customHeight="1" s="18">
@@ -4943,7 +4959,7 @@
         </is>
       </c>
       <c r="U50" s="42" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
     </row>
     <row r="51" ht="45" customHeight="1" s="18">
@@ -5048,13 +5064,13 @@
         </is>
       </c>
       <c r="U51" s="46" t="n">
-        <v>22</v>
+        <v>78</v>
       </c>
     </row>
     <row r="52" ht="45" customHeight="1" s="18">
       <c r="A52" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">DCGS </t>
+          <t>DCGS</t>
         </is>
       </c>
       <c r="B52" s="40" t="inlineStr">
@@ -5153,7 +5169,7 @@
         </is>
       </c>
       <c r="U52" s="42" t="n">
-        <v>64</v>
+        <v>117</v>
       </c>
     </row>
     <row r="53" ht="45" customHeight="1" s="18">
@@ -5259,7 +5275,7 @@
         </is>
       </c>
       <c r="U53" s="46" t="n">
-        <v>49</v>
+        <v>64</v>
       </c>
     </row>
     <row r="54" ht="45" customHeight="1" s="18">
@@ -5364,7 +5380,7 @@
         </is>
       </c>
       <c r="U54" s="42" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
     </row>
     <row r="55" ht="45" customHeight="1" s="18">
@@ -5469,7 +5485,7 @@
         </is>
       </c>
       <c r="U55" s="46" t="n">
-        <v>51</v>
+        <v>69</v>
       </c>
     </row>
     <row r="56" ht="45" customHeight="1" s="18">
@@ -5571,7 +5587,9 @@
           <t>2/5</t>
         </is>
       </c>
-      <c r="U56" s="42" t="n"/>
+      <c r="U56" s="42" t="n">
+        <v>66</v>
+      </c>
     </row>
     <row r="57" ht="45" customHeight="1" s="18">
       <c r="A57" s="43" t="inlineStr">
@@ -5675,7 +5693,7 @@
         </is>
       </c>
       <c r="U57" s="46" t="n">
-        <v>79</v>
+        <v>107</v>
       </c>
     </row>
     <row r="58" ht="45" customHeight="1" s="18">
@@ -5780,7 +5798,7 @@
         </is>
       </c>
       <c r="U58" s="42" t="n">
-        <v>47</v>
+        <v>62</v>
       </c>
     </row>
     <row r="59" ht="45" customHeight="1" s="18">
@@ -5796,7 +5814,7 @@
       </c>
       <c r="C59" s="44" t="inlineStr">
         <is>
-          <t>PMID: 38437548</t>
+          <t>PMID: 38437548</t>
         </is>
       </c>
       <c r="D59" s="45" t="inlineStr">
@@ -5885,7 +5903,7 @@
         </is>
       </c>
       <c r="U59" s="46" t="n">
-        <v>52</v>
+        <v>68</v>
       </c>
     </row>
     <row r="60" ht="45" customHeight="1" s="18">
@@ -5990,7 +6008,7 @@
         </is>
       </c>
       <c r="U60" s="42" t="n">
-        <v>57</v>
+        <v>110</v>
       </c>
     </row>
     <row r="61" ht="45" customHeight="1" s="18">
@@ -6093,7 +6111,7 @@
         </is>
       </c>
       <c r="U61" s="46" t="n">
-        <v>45</v>
+        <v>56</v>
       </c>
     </row>
     <row r="62" ht="45" customHeight="1" s="18">
@@ -6198,7 +6216,7 @@
         </is>
       </c>
       <c r="U62" s="42" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
     </row>
     <row r="63" ht="45" customHeight="1" s="18">
@@ -6303,7 +6321,7 @@
         </is>
       </c>
       <c r="U63" s="46" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="64" ht="45" customHeight="1" s="18">
@@ -6405,7 +6423,9 @@
           <t>2/5</t>
         </is>
       </c>
-      <c r="U64" s="42" t="n"/>
+      <c r="U64" s="42" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="65" ht="78" customHeight="1" s="18">
       <c r="A65" s="43" t="inlineStr">
@@ -6510,7 +6530,7 @@
         </is>
       </c>
       <c r="U65" s="46" t="n">
-        <v>58</v>
+        <v>109</v>
       </c>
     </row>
     <row r="66" ht="65" customHeight="1" s="18">
@@ -6617,7 +6637,7 @@
         </is>
       </c>
       <c r="U66" s="42" t="n">
-        <v>32</v>
+        <v>74</v>
       </c>
     </row>
     <row r="67" ht="78" customHeight="1" s="18">
@@ -6722,7 +6742,7 @@
         </is>
       </c>
       <c r="U67" s="46" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="68" ht="65" customHeight="1" s="18">
@@ -6827,7 +6847,7 @@
         </is>
       </c>
       <c r="U68" s="42" t="n">
-        <v>29</v>
+        <v>65</v>
       </c>
     </row>
     <row r="69" ht="52" customHeight="1" s="18">
@@ -6843,7 +6863,7 @@
       </c>
       <c r="C69" s="44" t="inlineStr">
         <is>
-          <t>PMID: 41331466; DOI: 10.1186/s13059-025-03876-0</t>
+          <t>PMID: 41331466</t>
         </is>
       </c>
       <c r="D69" s="45" t="inlineStr">
@@ -6932,7 +6952,7 @@
         </is>
       </c>
       <c r="U69" s="46" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
     </row>
     <row r="70" ht="78" customHeight="1" s="18">
@@ -7037,7 +7057,7 @@
         </is>
       </c>
       <c r="U70" s="42" t="n">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="71" ht="65" customHeight="1" s="18">
@@ -7053,7 +7073,7 @@
       </c>
       <c r="C71" s="44" t="inlineStr">
         <is>
-          <t>PMID: 41639465; DOI: 10.1038/s41586-025-09989-7</t>
+          <t>PMID: 41639465</t>
         </is>
       </c>
       <c r="D71" s="45" t="inlineStr">
@@ -7142,7 +7162,7 @@
         </is>
       </c>
       <c r="U71" s="46" t="n">
-        <v>28</v>
+        <v>57</v>
       </c>
     </row>
     <row r="72" ht="65" customHeight="1" s="18">
@@ -7244,7 +7264,9 @@
           <t>4/5</t>
         </is>
       </c>
-      <c r="U72" s="42" t="n"/>
+      <c r="U72" s="42" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="43" t="inlineStr">
@@ -7348,26 +7370,26 @@
         </is>
       </c>
       <c r="U73" s="46" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A7:R7"/>
+    <mergeCell ref="A4:U4"/>
+    <mergeCell ref="A2:U2"/>
     <mergeCell ref="H12:M12"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A7:U7"/>
     <mergeCell ref="A12:D12"/>
-    <mergeCell ref="Q12:R12"/>
-    <mergeCell ref="A10:R10"/>
+    <mergeCell ref="S12:T12"/>
+    <mergeCell ref="A10:U10"/>
+    <mergeCell ref="A5:U5"/>
     <mergeCell ref="E12:G12"/>
-    <mergeCell ref="A1:R1"/>
-    <mergeCell ref="A5:R5"/>
-    <mergeCell ref="A9:R9"/>
-    <mergeCell ref="A8:R8"/>
-    <mergeCell ref="A6:R6"/>
-    <mergeCell ref="A4:R4"/>
+    <mergeCell ref="N12:Q12"/>
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A9:U9"/>
+    <mergeCell ref="A8:U8"/>
+    <mergeCell ref="A3:U3"/>
+    <mergeCell ref="A6:U6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>

</xml_diff>